<commit_message>
refactor(data & rpa): unify sample_data across root, backend, and docs, and enhance RPA bot path resolution
</commit_message>
<xml_diff>
--- a/backend/sample_data/01_Fresh_Admissions_Bulk_Upload.xlsx
+++ b/backend/sample_data/01_Fresh_Admissions_Bulk_Upload.xlsx
@@ -468,12 +468,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aditya Verma</t>
+          <t>Aarav Roy</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>aditya.verma.2026@university.edu</t>
+          <t>aarav.roy.test2026@university.edu</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -491,12 +491,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>9822334401</t>
+          <t>9822001101</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>404 Tech Park, Bengaluru, Karnataka</t>
+          <t>404 Cyber City, Bengaluru, Karnataka</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pooja.hegde.2026@university.edu</t>
+          <t>pooja.hegde.test2026@university.edu</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>9822334402</t>
+          <t>9822001102</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>nikhil.chopra.2026@university.edu</t>
+          <t>nikhil.chopra.test2026@university.edu</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>9822334403</t>
+          <t>9822001103</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>anjali.deshmukh.2026@university.edu</t>
+          <t>anjali.deshmukh.test2026@university.edu</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>9822334404</t>
+          <t>9822001104</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>siddharth.sen.2026@university.edu</t>
+          <t>siddharth.sen.test2026@university.edu</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>9822334405</t>
+          <t>9822001105</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>kavita.pillai.2026@university.edu</t>
+          <t>kavita.pillai.test2026@university.edu</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>9822334406</t>
+          <t>9822001106</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>varun.grover.2026@university.edu</t>
+          <t>varun.grover.test2026@university.edu</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>9822334407</t>
+          <t>9822001107</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>sneha.kulkarni.2026@university.edu</t>
+          <t>sneha.kulkarni.test2026@university.edu</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9822334408</t>
+          <t>9822001108</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">

</xml_diff>